<commit_message>
Adding new items from recent streams.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-02/P1012202501-BOM V2.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-02/P1012202501-BOM V2.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">Project:</t>
   </si>
   <si>
-    <t xml:space="preserve">P1012202501-01</t>
+    <t xml:space="preserve">P1012202501-02</t>
   </si>
   <si>
     <t xml:space="preserve">Per board LV Cost</t>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">187-CL31B106KBHNNNE</t>
   </si>
   <si>
-    <t xml:space="preserve">C5,C6,C11,C12,C15,C18,C20,C23,C24,C25,C28</t>
+    <t xml:space="preserve">C5,C6,C11,C12,C15,C18,C20,C23,C24,C25,C28,C30</t>
   </si>
   <si>
     <t xml:space="preserve">CC0603104050AAAX7R</t>
@@ -676,7 +676,7 @@
     <t xml:space="preserve">710-435151014845</t>
   </si>
   <si>
-    <t xml:space="preserve">TP1,TP2,TP3,TP4,TP5,TP6,TP7,TP10,TP11,TP12,TP13,TP14,TP15,TP16,TP17,TP18,TP19,TP20,TP21,TP22,TP23,TP24,TP25</t>
+    <t xml:space="preserve">TP1,TP2,TP3,TP4,TP5,TP6,TP7,TP10,TP11,TP12,TP13,TP14,TP15,TP16,TP17,TP18,TP19,TP20,TP21,TP22,TP23,TP24,TP25,TP26,TP27,TP28,TP29,TP30,TP31,TP32,TP33,TP34,TP35,TP36</t>
   </si>
   <si>
     <t xml:space="preserve">TP5010</t>
@@ -691,7 +691,7 @@
     <t xml:space="preserve">PCB</t>
   </si>
   <si>
-    <t xml:space="preserve">P1012202501-PCB-01</t>
+    <t xml:space="preserve">P1012202501-PCB-02</t>
   </si>
   <si>
     <t xml:space="preserve">Jumper for J1, J2, and J3</t>
@@ -891,40 +891,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1114,2361 +1118,2361 @@
   <dimension ref="A1:P59"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="4.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="31.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="17.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="109.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="31.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="16.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="20.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="16.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" s="2" t="n">
         <f aca="false">SUM(I6:I61)</f>
-        <v>77.98</v>
-      </c>
-      <c r="J1" s="1" t="s">
+        <v>82.37</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" s="2" t="n">
         <f aca="false">SUM(K6:K56)</f>
-        <v>25.999</v>
+        <v>28.455</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="4" t="n">
-        <v>1</v>
+      <c r="B2" s="3"/>
+      <c r="C2" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="5" t="s">
+      <c r="N5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="O5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="P5" s="5" t="s">
+      <c r="P5" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="3" t="s">
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <v>0.22</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="8" t="n">
         <f aca="false">B6*H6</f>
         <v>0.88</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v>0.068</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="K6" s="8" t="n">
         <f aca="false">B6*J6</f>
         <v>0.272</v>
       </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="3" t="s">
+      <c r="F7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="8" t="n">
         <f aca="false">B7*H7</f>
-        <v>1.1</v>
-      </c>
-      <c r="J7" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J7" s="8" t="n">
         <v>0.012</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K7" s="8" t="n">
         <f aca="false">B7*J7</f>
-        <v>0.132</v>
-      </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
+        <v>0.144</v>
+      </c>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="F8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="8" t="n">
         <v>0.6</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="8" t="n">
         <f aca="false">B8*H8</f>
         <v>2.4</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="8" t="n">
         <v>0.187</v>
       </c>
-      <c r="K8" s="7" t="n">
+      <c r="K8" s="8" t="n">
         <f aca="false">B8*J8</f>
         <v>0.748</v>
       </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="3" t="s">
+      <c r="F9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="8" t="n">
         <f aca="false">B9*H9</f>
         <v>0.5</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="J9" s="8" t="n">
         <v>0.023</v>
       </c>
-      <c r="K9" s="7" t="n">
+      <c r="K9" s="8" t="n">
         <f aca="false">B9*J9</f>
         <v>0.115</v>
       </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="3" t="s">
+      <c r="F10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I10" s="8" t="n">
         <f aca="false">B10*H10</f>
         <v>0.2</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="8" t="n">
         <v>0.043</v>
       </c>
-      <c r="K10" s="7" t="n">
+      <c r="K10" s="8" t="n">
         <f aca="false">B10*J10</f>
         <v>0.086</v>
       </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="3" t="s">
+      <c r="F11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="8" t="n">
         <v>1.49</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="8" t="n">
         <f aca="false">B11*H11</f>
         <v>1.49</v>
       </c>
-      <c r="J11" s="7" t="n">
+      <c r="J11" s="8" t="n">
         <v>0.472</v>
       </c>
-      <c r="K11" s="7" t="n">
+      <c r="K11" s="8" t="n">
         <f aca="false">B11*J11</f>
         <v>0.472</v>
       </c>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" s="3" t="s">
+      <c r="F12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I12" s="7" t="n">
+      <c r="I12" s="8" t="n">
         <f aca="false">B12*H12</f>
         <v>0.1</v>
       </c>
-      <c r="J12" s="7" t="n">
+      <c r="J12" s="8" t="n">
         <v>0.019</v>
       </c>
-      <c r="K12" s="7" t="n">
+      <c r="K12" s="8" t="n">
         <f aca="false">B12*J12</f>
         <v>0.019</v>
       </c>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="B13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="3" t="s">
+      <c r="F13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="I13" s="7" t="n">
+      <c r="I13" s="8" t="n">
         <f aca="false">B13*H13</f>
         <v>0.15</v>
       </c>
-      <c r="J13" s="7" t="n">
+      <c r="J13" s="8" t="n">
         <v>0.035</v>
       </c>
-      <c r="K13" s="7" t="n">
+      <c r="K13" s="8" t="n">
         <f aca="false">B13*J13</f>
         <v>0.035</v>
       </c>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="B14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="3" t="s">
+      <c r="F14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="I14" s="7" t="n">
+      <c r="I14" s="8" t="n">
         <f aca="false">B14*H14</f>
         <v>0.33</v>
       </c>
-      <c r="J14" s="7" t="n">
+      <c r="J14" s="8" t="n">
         <v>0.128</v>
       </c>
-      <c r="K14" s="7" t="n">
+      <c r="K14" s="8" t="n">
         <f aca="false">B14*J14</f>
         <v>0.128</v>
       </c>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="B15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="3" t="s">
+      <c r="F15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="8" t="n">
         <v>0.48</v>
       </c>
-      <c r="I15" s="7" t="n">
+      <c r="I15" s="8" t="n">
         <f aca="false">B15*H15</f>
         <v>0.48</v>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="J15" s="8" t="n">
         <v>0.189</v>
       </c>
-      <c r="K15" s="7" t="n">
+      <c r="K15" s="8" t="n">
         <f aca="false">B15*J15</f>
         <v>0.189</v>
       </c>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="3" t="s">
+      <c r="F16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H16" s="8" t="n">
         <v>0.62</v>
       </c>
-      <c r="I16" s="7" t="n">
+      <c r="I16" s="8" t="n">
         <f aca="false">B16*H16</f>
         <v>1.86</v>
       </c>
-      <c r="J16" s="7" t="n">
+      <c r="J16" s="8" t="n">
         <v>0.246</v>
       </c>
-      <c r="K16" s="7" t="n">
+      <c r="K16" s="8" t="n">
         <f aca="false">B16*J16</f>
         <v>0.738</v>
       </c>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="B17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="3" t="s">
+      <c r="F17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="H17" s="8" t="n">
         <v>0.78</v>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="8" t="n">
         <f aca="false">B17*H17</f>
         <v>0.78</v>
       </c>
-      <c r="J17" s="7" t="n">
+      <c r="J17" s="8" t="n">
         <v>0.484</v>
       </c>
-      <c r="K17" s="7" t="n">
+      <c r="K17" s="8" t="n">
         <f aca="false">B17*J17</f>
         <v>0.484</v>
       </c>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="B18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G18" s="3" t="s">
+      <c r="F18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="H18" s="8" t="n">
         <v>0.79</v>
       </c>
-      <c r="I18" s="7" t="n">
+      <c r="I18" s="8" t="n">
         <f aca="false">B18*H18</f>
         <v>0.79</v>
       </c>
-      <c r="J18" s="7" t="n">
+      <c r="J18" s="8" t="n">
         <v>0.369</v>
       </c>
-      <c r="K18" s="7" t="n">
+      <c r="K18" s="8" t="n">
         <f aca="false">B18*J18</f>
         <v>0.369</v>
       </c>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" s="3" t="s">
+      <c r="F19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="7" t="n">
+      <c r="H19" s="8" t="n">
         <v>0.27</v>
       </c>
-      <c r="I19" s="7" t="n">
+      <c r="I19" s="8" t="n">
         <f aca="false">B19*H19</f>
         <v>0.54</v>
       </c>
-      <c r="J19" s="7" t="n">
+      <c r="J19" s="8" t="n">
         <v>0.049</v>
       </c>
-      <c r="K19" s="7" t="n">
+      <c r="K19" s="8" t="n">
         <f aca="false">B19*J19</f>
         <v>0.098</v>
       </c>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="B20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="3" t="s">
+      <c r="F20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H20" s="8" t="n">
         <v>0.36</v>
       </c>
-      <c r="I20" s="7" t="n">
+      <c r="I20" s="8" t="n">
         <f aca="false">B20*H20</f>
         <v>0.36</v>
       </c>
-      <c r="J20" s="7" t="n">
+      <c r="J20" s="8" t="n">
         <v>0.076</v>
       </c>
-      <c r="K20" s="7" t="n">
+      <c r="K20" s="8" t="n">
         <f aca="false">B20*J20</f>
         <v>0.076</v>
       </c>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="3" t="s">
+      <c r="F21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="H21" s="7" t="n">
+      <c r="H21" s="8" t="n">
         <v>1.11</v>
       </c>
-      <c r="I21" s="7" t="n">
+      <c r="I21" s="8" t="n">
         <f aca="false">B21*H21</f>
         <v>5.55</v>
       </c>
-      <c r="J21" s="7" t="n">
+      <c r="J21" s="8" t="n">
         <v>0.343</v>
       </c>
-      <c r="K21" s="7" t="n">
+      <c r="K21" s="8" t="n">
         <f aca="false">B21*J21</f>
         <v>1.715</v>
       </c>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="3"/>
-      <c r="P21" s="3"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="3" t="s">
+      <c r="B22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="3" t="s">
+      <c r="F22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="H22" s="7" t="n">
+      <c r="H22" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="I22" s="7" t="n">
+      <c r="I22" s="8" t="n">
         <f aca="false">B22*H22</f>
         <v>0.15</v>
       </c>
-      <c r="J22" s="7" t="n">
+      <c r="J22" s="8" t="n">
         <v>0.045</v>
       </c>
-      <c r="K22" s="7" t="n">
+      <c r="K22" s="8" t="n">
         <f aca="false">B22*J22</f>
         <v>0.045</v>
       </c>
-      <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="3"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B23" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="3" t="s">
+      <c r="F23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="H23" s="7" t="n">
+      <c r="H23" s="8" t="n">
         <v>0.71</v>
       </c>
-      <c r="I23" s="7" t="n">
+      <c r="I23" s="8" t="n">
         <f aca="false">B23*H23</f>
         <v>0.71</v>
       </c>
-      <c r="J23" s="7" t="n">
+      <c r="J23" s="8" t="n">
         <v>0.342</v>
       </c>
-      <c r="K23" s="7" t="n">
+      <c r="K23" s="8" t="n">
         <f aca="false">B23*J23</f>
         <v>0.342</v>
       </c>
-      <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
-      <c r="P23" s="3"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="B24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="F24" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G24" s="3" t="s">
+      <c r="F24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="H24" s="7" t="n">
+      <c r="H24" s="8" t="n">
         <v>0.71</v>
       </c>
-      <c r="I24" s="7" t="n">
+      <c r="I24" s="8" t="n">
         <f aca="false">B24*H24</f>
         <v>0.71</v>
       </c>
-      <c r="J24" s="7" t="n">
+      <c r="J24" s="8" t="n">
         <v>0.342</v>
       </c>
-      <c r="K24" s="7" t="n">
+      <c r="K24" s="8" t="n">
         <f aca="false">B24*J24</f>
         <v>0.342</v>
       </c>
-      <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="3"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="3" t="s">
+      <c r="B25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="3" t="s">
+      <c r="F25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="H25" s="7" t="n">
+      <c r="H25" s="8" t="n">
         <v>6.71</v>
       </c>
-      <c r="I25" s="7" t="n">
+      <c r="I25" s="8" t="n">
         <f aca="false">B25*H25</f>
         <v>6.71</v>
       </c>
-      <c r="J25" s="7" t="n">
+      <c r="J25" s="8" t="n">
         <v>3.98</v>
       </c>
-      <c r="K25" s="7" t="n">
+      <c r="K25" s="8" t="n">
         <f aca="false">B25*J25</f>
         <v>3.98</v>
       </c>
-      <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
-      <c r="N25" s="3"/>
-      <c r="O25" s="3"/>
-      <c r="P25" s="3"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="3" t="s">
+      <c r="B26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="F26" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G26" s="3" t="s">
+      <c r="F26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="H26" s="7" t="n">
+      <c r="H26" s="8" t="n">
         <v>0.81</v>
       </c>
-      <c r="I26" s="7" t="n">
+      <c r="I26" s="8" t="n">
         <f aca="false">B26*H26</f>
         <v>0.81</v>
       </c>
-      <c r="J26" s="7" t="n">
+      <c r="J26" s="8" t="n">
         <v>0.38</v>
       </c>
-      <c r="K26" s="7" t="n">
+      <c r="K26" s="8" t="n">
         <f aca="false">B26*J26</f>
         <v>0.38</v>
       </c>
-      <c r="L26" s="3" t="s">
+      <c r="L26" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="M26" s="3" t="s">
+      <c r="M26" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="N26" s="3" t="n">
+      <c r="N26" s="4" t="n">
         <v>0.39507</v>
       </c>
-      <c r="O26" s="3" t="n">
+      <c r="O26" s="4" t="n">
         <v>0.81</v>
       </c>
-      <c r="P26" s="3"/>
+      <c r="P26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="3" t="s">
+      <c r="B27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G27" s="3" t="s">
+      <c r="F27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="H27" s="7" t="n">
+      <c r="H27" s="8" t="n">
         <v>3.55</v>
       </c>
-      <c r="I27" s="7" t="n">
+      <c r="I27" s="8" t="n">
         <f aca="false">B27*H27</f>
         <v>3.55</v>
       </c>
-      <c r="J27" s="7" t="n">
+      <c r="J27" s="8" t="n">
         <v>1.31</v>
       </c>
-      <c r="K27" s="7" t="n">
+      <c r="K27" s="8" t="n">
         <f aca="false">B27*J27</f>
         <v>1.31</v>
       </c>
-      <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="3"/>
-      <c r="P27" s="3"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="3" t="s">
+      <c r="B28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G28" s="3" t="s">
+      <c r="F28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="H28" s="7" t="n">
+      <c r="H28" s="8" t="n">
         <v>3.52</v>
       </c>
-      <c r="I28" s="7" t="n">
+      <c r="I28" s="8" t="n">
         <f aca="false">B28*H28</f>
         <v>3.52</v>
       </c>
-      <c r="J28" s="7" t="n">
+      <c r="J28" s="8" t="n">
         <v>2.13</v>
       </c>
-      <c r="K28" s="7" t="n">
+      <c r="K28" s="8" t="n">
         <f aca="false">B28*J28</f>
         <v>2.13</v>
       </c>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="3"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="3" t="s">
+      <c r="B29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G29" s="3" t="s">
+      <c r="F29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="H29" s="7" t="n">
+      <c r="H29" s="8" t="n">
         <v>1.89</v>
       </c>
-      <c r="I29" s="7" t="n">
+      <c r="I29" s="8" t="n">
         <f aca="false">B29*H29</f>
         <v>1.89</v>
       </c>
-      <c r="J29" s="7" t="n">
+      <c r="J29" s="8" t="n">
         <v>1.22</v>
       </c>
-      <c r="K29" s="7" t="n">
+      <c r="K29" s="8" t="n">
         <f aca="false">B29*J29</f>
         <v>1.22</v>
       </c>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="N29" s="3"/>
-      <c r="O29" s="3"/>
-      <c r="P29" s="3"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="F30" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G30" s="3" t="s">
+      <c r="F30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="H30" s="7" t="n">
+      <c r="H30" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I30" s="7" t="n">
+      <c r="I30" s="8" t="n">
         <f aca="false">B30*H30</f>
         <v>0.3</v>
       </c>
-      <c r="J30" s="7" t="n">
+      <c r="J30" s="8" t="n">
         <v>0.071</v>
       </c>
-      <c r="K30" s="7" t="n">
+      <c r="K30" s="8" t="n">
         <f aca="false">B30*J30</f>
         <v>0.213</v>
       </c>
-      <c r="L30" s="3"/>
-      <c r="M30" s="3"/>
-      <c r="N30" s="3"/>
-      <c r="O30" s="3"/>
-      <c r="P30" s="3"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
+      <c r="P30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B31" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="B31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="F31" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G31" s="3" t="s">
+      <c r="F31" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="7" t="n">
+      <c r="H31" s="8" t="n">
         <v>0.17</v>
       </c>
-      <c r="I31" s="7" t="n">
+      <c r="I31" s="8" t="n">
         <f aca="false">B31*H31</f>
         <v>0.17</v>
       </c>
-      <c r="J31" s="7" t="n">
+      <c r="J31" s="8" t="n">
         <v>0.163</v>
       </c>
-      <c r="K31" s="7" t="n">
+      <c r="K31" s="8" t="n">
         <f aca="false">B31*J31</f>
         <v>0.163</v>
       </c>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
-      <c r="N31" s="3"/>
-      <c r="O31" s="3"/>
-      <c r="P31" s="3"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+      <c r="P31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="F32" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G32" s="3" t="s">
+      <c r="F32" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="H32" s="7" t="n">
+      <c r="H32" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="I32" s="7" t="n">
+      <c r="I32" s="8" t="n">
         <f aca="false">B32*H32</f>
         <v>0.66</v>
       </c>
-      <c r="J32" s="7" t="n">
+      <c r="J32" s="8" t="n">
         <v>0.199</v>
       </c>
-      <c r="K32" s="7" t="n">
+      <c r="K32" s="8" t="n">
         <f aca="false">B32*J32</f>
         <v>0.398</v>
       </c>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
-      <c r="N32" s="3"/>
-      <c r="O32" s="3"/>
-      <c r="P32" s="3"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F33" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G33" s="3" t="s">
+      <c r="F33" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="H33" s="7" t="n">
+      <c r="H33" s="8" t="n">
         <v>0.76</v>
       </c>
-      <c r="I33" s="7" t="n">
+      <c r="I33" s="8" t="n">
         <f aca="false">B33*H33</f>
         <v>4.56</v>
       </c>
-      <c r="J33" s="7" t="n">
+      <c r="J33" s="8" t="n">
         <v>0.303</v>
       </c>
-      <c r="K33" s="7" t="n">
+      <c r="K33" s="8" t="n">
         <f aca="false">B33*J33</f>
         <v>1.818</v>
       </c>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="3"/>
-      <c r="O33" s="3"/>
-      <c r="P33" s="3"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B34" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="B34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="F34" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G34" s="3" t="s">
+      <c r="F34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="H34" s="7" t="n">
+      <c r="H34" s="8" t="n">
         <v>0.14</v>
       </c>
-      <c r="I34" s="7" t="n">
+      <c r="I34" s="8" t="n">
         <f aca="false">B34*H34</f>
         <v>0.14</v>
       </c>
-      <c r="J34" s="7" t="n">
+      <c r="J34" s="8" t="n">
         <v>0.42</v>
       </c>
-      <c r="K34" s="7" t="n">
+      <c r="K34" s="8" t="n">
         <f aca="false">B34*J34</f>
         <v>0.42</v>
       </c>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
-      <c r="O34" s="3"/>
-      <c r="P34" s="3"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="F35" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G35" s="3" t="s">
+      <c r="F35" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="H35" s="7" t="n">
+      <c r="H35" s="8" t="n">
         <v>0.19</v>
       </c>
-      <c r="I35" s="7" t="n">
+      <c r="I35" s="8" t="n">
         <f aca="false">B35*H35</f>
         <v>0.38</v>
       </c>
-      <c r="J35" s="7" t="n">
+      <c r="J35" s="8" t="n">
         <v>0.015</v>
       </c>
-      <c r="K35" s="7" t="n">
+      <c r="K35" s="8" t="n">
         <f aca="false">B35*J35</f>
         <v>0.03</v>
       </c>
-      <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
-      <c r="N35" s="3"/>
-      <c r="O35" s="3"/>
-      <c r="P35" s="3"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+      <c r="P35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="B36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="3" t="s">
+      <c r="B36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="F36" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G36" s="3" t="s">
+      <c r="F36" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G36" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="H36" s="7" t="n">
+      <c r="H36" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I36" s="7" t="n">
+      <c r="I36" s="8" t="n">
         <f aca="false">B36*H36</f>
         <v>0.1</v>
       </c>
-      <c r="J36" s="7" t="n">
+      <c r="J36" s="8" t="n">
         <v>0.021</v>
       </c>
-      <c r="K36" s="7" t="n">
+      <c r="K36" s="8" t="n">
         <f aca="false">B36*J36</f>
         <v>0.021</v>
       </c>
-      <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
-      <c r="N36" s="3"/>
-      <c r="O36" s="3"/>
-      <c r="P36" s="3"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+      <c r="P36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="3" t="s">
+      <c r="B37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F37" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G37" s="3" t="s">
+      <c r="F37" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H37" s="7" t="n">
+      <c r="H37" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I37" s="7" t="n">
+      <c r="I37" s="8" t="n">
         <f aca="false">B37*H37</f>
         <v>0.1</v>
       </c>
-      <c r="J37" s="7" t="n">
+      <c r="J37" s="8" t="n">
         <v>0.043</v>
       </c>
-      <c r="K37" s="7" t="n">
+      <c r="K37" s="8" t="n">
         <f aca="false">B37*J37</f>
         <v>0.043</v>
       </c>
-      <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
-      <c r="N37" s="3"/>
-      <c r="O37" s="3"/>
-      <c r="P37" s="3"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F38" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G38" s="3" t="s">
+      <c r="F38" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="H38" s="7" t="n">
+      <c r="H38" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="I38" s="7" t="n">
+      <c r="I38" s="8" t="n">
         <f aca="false">B38*H38</f>
         <v>1.32</v>
       </c>
-      <c r="J38" s="7" t="n">
+      <c r="J38" s="8" t="n">
         <v>0.031</v>
       </c>
-      <c r="K38" s="7" t="n">
+      <c r="K38" s="8" t="n">
         <f aca="false">B38*J38</f>
         <v>0.372</v>
       </c>
-      <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
-      <c r="N38" s="3"/>
-      <c r="O38" s="3"/>
-      <c r="P38" s="3"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="4"/>
+      <c r="O38" s="4"/>
+      <c r="P38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="B39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3" t="s">
+      <c r="B39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F39" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G39" s="3" t="s">
+      <c r="F39" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G39" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="H39" s="7" t="n">
+      <c r="H39" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I39" s="7" t="n">
+      <c r="I39" s="8" t="n">
         <f aca="false">B39*H39</f>
         <v>0.1</v>
       </c>
-      <c r="J39" s="7" t="n">
+      <c r="J39" s="8" t="n">
         <v>0.013</v>
       </c>
-      <c r="K39" s="7" t="n">
+      <c r="K39" s="8" t="n">
         <f aca="false">B39*J39</f>
         <v>0.013</v>
       </c>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
-      <c r="N39" s="3"/>
-      <c r="O39" s="3"/>
-      <c r="P39" s="3"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="F40" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G40" s="3" t="s">
+      <c r="F40" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="H40" s="7" t="n">
+      <c r="H40" s="8" t="n">
         <v>0.12</v>
       </c>
-      <c r="I40" s="7" t="n">
+      <c r="I40" s="8" t="n">
         <f aca="false">B40*H40</f>
         <v>0.72</v>
       </c>
-      <c r="J40" s="7" t="n">
+      <c r="J40" s="8" t="n">
         <v>0.041</v>
       </c>
-      <c r="K40" s="7" t="n">
+      <c r="K40" s="8" t="n">
         <f aca="false">B40*J40</f>
         <v>0.246</v>
       </c>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
-      <c r="N40" s="3"/>
-      <c r="O40" s="3"/>
-      <c r="P40" s="3"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B41" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="3" t="s">
+      <c r="B41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="F41" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G41" s="3" t="s">
+      <c r="F41" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G41" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="H41" s="7" t="n">
+      <c r="H41" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="I41" s="7" t="n">
+      <c r="I41" s="8" t="n">
         <f aca="false">B41*H41</f>
         <v>0.11</v>
       </c>
-      <c r="J41" s="7" t="n">
+      <c r="J41" s="8" t="n">
         <v>0.009</v>
       </c>
-      <c r="K41" s="7" t="n">
+      <c r="K41" s="8" t="n">
         <f aca="false">B41*J41</f>
         <v>0.009</v>
       </c>
-      <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
-      <c r="N41" s="3"/>
-      <c r="O41" s="3"/>
-      <c r="P41" s="3"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="B42" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="3" t="s">
+      <c r="B42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="F42" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G42" s="3" t="s">
+      <c r="F42" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G42" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="H42" s="7" t="n">
+      <c r="H42" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I42" s="7" t="n">
+      <c r="I42" s="8" t="n">
         <f aca="false">B42*H42</f>
         <v>0.1</v>
       </c>
-      <c r="J42" s="7" t="n">
+      <c r="J42" s="8" t="n">
         <v>0.042</v>
       </c>
-      <c r="K42" s="7" t="n">
+      <c r="K42" s="8" t="n">
         <f aca="false">B42*J42</f>
         <v>0.042</v>
       </c>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
-      <c r="N42" s="3"/>
-      <c r="O42" s="3"/>
-      <c r="P42" s="3"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="F43" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G43" s="3" t="s">
+      <c r="F43" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G43" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="H43" s="7" t="n">
+      <c r="H43" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="I43" s="7" t="n">
+      <c r="I43" s="8" t="n">
         <f aca="false">B43*H43</f>
         <v>0.22</v>
       </c>
-      <c r="J43" s="7" t="n">
+      <c r="J43" s="8" t="n">
         <v>0.031</v>
       </c>
-      <c r="K43" s="7" t="n">
+      <c r="K43" s="8" t="n">
         <f aca="false">B43*J43</f>
         <v>0.062</v>
       </c>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
-      <c r="N43" s="3"/>
-      <c r="O43" s="3"/>
-      <c r="P43" s="3"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
+      <c r="P43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="B44" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="3" t="s">
+      <c r="B44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="F44" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G44" s="3" t="s">
+      <c r="F44" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G44" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="H44" s="7" t="n">
+      <c r="H44" s="8" t="n">
         <v>0.24</v>
       </c>
-      <c r="I44" s="7" t="n">
+      <c r="I44" s="8" t="n">
         <f aca="false">B44*H44</f>
         <v>0.24</v>
       </c>
-      <c r="J44" s="7" t="n">
+      <c r="J44" s="8" t="n">
         <v>0.139</v>
       </c>
-      <c r="K44" s="7" t="n">
+      <c r="K44" s="8" t="n">
         <f aca="false">B44*J44</f>
         <v>0.139</v>
       </c>
-      <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
-      <c r="N44" s="3"/>
-      <c r="O44" s="3"/>
-      <c r="P44" s="3"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="F45" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G45" s="3" t="s">
+      <c r="F45" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G45" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="H45" s="7" t="n">
+      <c r="H45" s="8" t="n">
         <v>0.17</v>
       </c>
-      <c r="I45" s="7" t="n">
+      <c r="I45" s="8" t="n">
         <f aca="false">B45*H45</f>
         <v>0.34</v>
       </c>
-      <c r="J45" s="7" t="n">
+      <c r="J45" s="8" t="n">
         <v>0.051</v>
       </c>
-      <c r="K45" s="7" t="n">
+      <c r="K45" s="8" t="n">
         <f aca="false">B45*J45</f>
         <v>0.102</v>
       </c>
-      <c r="L45" s="3"/>
-      <c r="M45" s="3"/>
-      <c r="N45" s="3"/>
-      <c r="O45" s="3"/>
-      <c r="P45" s="3"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B46" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="3" t="s">
+      <c r="B46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="F46" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G46" s="3" t="s">
+      <c r="F46" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G46" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="H46" s="7" t="n">
+      <c r="H46" s="8" t="n">
         <v>0.14</v>
       </c>
-      <c r="I46" s="7" t="n">
+      <c r="I46" s="8" t="n">
         <f aca="false">B46*H46</f>
         <v>0.14</v>
       </c>
-      <c r="J46" s="7" t="n">
+      <c r="J46" s="8" t="n">
         <v>0.052</v>
       </c>
-      <c r="K46" s="7" t="n">
+      <c r="K46" s="8" t="n">
         <f aca="false">B46*J46</f>
         <v>0.052</v>
       </c>
-      <c r="L46" s="3"/>
-      <c r="M46" s="3"/>
-      <c r="N46" s="3"/>
-      <c r="O46" s="3"/>
-      <c r="P46" s="3"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B47" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" s="3" t="s">
+      <c r="B47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="F47" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G47" s="3" t="s">
+      <c r="F47" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G47" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="H47" s="7" t="n">
+      <c r="H47" s="8" t="n">
         <v>0.17</v>
       </c>
-      <c r="I47" s="7" t="n">
+      <c r="I47" s="8" t="n">
         <f aca="false">B47*H47</f>
         <v>0.17</v>
       </c>
-      <c r="J47" s="7" t="n">
+      <c r="J47" s="8" t="n">
         <v>0.048</v>
       </c>
-      <c r="K47" s="7" t="n">
+      <c r="K47" s="8" t="n">
         <f aca="false">B47*J47</f>
         <v>0.048</v>
       </c>
-      <c r="L47" s="3"/>
-      <c r="M47" s="3"/>
-      <c r="N47" s="3"/>
-      <c r="O47" s="3"/>
-      <c r="P47" s="3"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+      <c r="P47" s="4"/>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D48" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E48" s="3" t="n">
+      <c r="E48" s="4" t="n">
         <v>435151014845</v>
       </c>
-      <c r="F48" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G48" s="3" t="s">
+      <c r="F48" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G48" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="H48" s="7" t="n">
+      <c r="H48" s="8" t="n">
         <v>0.54</v>
       </c>
-      <c r="I48" s="7" t="n">
+      <c r="I48" s="8" t="n">
         <f aca="false">B48*H48</f>
         <v>1.08</v>
       </c>
-      <c r="J48" s="7" t="n">
+      <c r="J48" s="8" t="n">
         <v>0.363</v>
       </c>
-      <c r="K48" s="7" t="n">
+      <c r="K48" s="8" t="n">
         <f aca="false">B48*J48</f>
         <v>0.726</v>
       </c>
-      <c r="L48" s="3"/>
-      <c r="M48" s="3"/>
-      <c r="N48" s="3"/>
-      <c r="O48" s="3"/>
-      <c r="P48" s="3"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="B49" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="C49" s="3" t="s">
+      <c r="B49" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D49" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="E49" s="3" t="n">
+      <c r="E49" s="4" t="n">
         <v>5010</v>
       </c>
-      <c r="F49" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G49" s="3" t="s">
+      <c r="F49" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G49" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="H49" s="7" t="n">
+      <c r="H49" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="I49" s="7" t="n">
+      <c r="I49" s="8" t="n">
         <f aca="false">B49*H49</f>
-        <v>7.59</v>
-      </c>
-      <c r="J49" s="7" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="J49" s="8" t="n">
         <v>0.188</v>
       </c>
-      <c r="K49" s="7" t="n">
+      <c r="K49" s="8" t="n">
         <f aca="false">B49*J49</f>
-        <v>4.324</v>
-      </c>
-      <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
-      <c r="N49" s="3"/>
-      <c r="O49" s="3"/>
-      <c r="P49" s="3"/>
+        <v>6.768</v>
+      </c>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
+      <c r="P49" s="4"/>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="B50" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" s="3" t="s">
+      <c r="B50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="7" t="n">
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I50" s="7" t="n">
+      <c r="I50" s="8" t="n">
         <f aca="false">B50*H50</f>
         <v>5</v>
       </c>
-      <c r="J50" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K50" s="7" t="n">
+      <c r="J50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="8" t="n">
         <f aca="false">B50*J50</f>
         <v>1</v>
       </c>
-      <c r="L50" s="3"/>
-      <c r="M50" s="3"/>
-      <c r="N50" s="3"/>
-      <c r="O50" s="3"/>
-      <c r="P50" s="3"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="4"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="E51" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="F51" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G51" s="8" t="s">
+      <c r="F51" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="H51" s="7" t="n">
+      <c r="H51" s="8" t="n">
         <v>0.23</v>
       </c>
-      <c r="I51" s="7" t="n">
+      <c r="I51" s="8" t="n">
         <f aca="false">B51*H51</f>
         <v>0.69</v>
       </c>
-      <c r="J51" s="7" t="n">
+      <c r="J51" s="8" t="n">
         <v>0.111</v>
       </c>
-      <c r="K51" s="7" t="n">
+      <c r="K51" s="8" t="n">
         <f aca="false">B51*J51</f>
         <v>0.333</v>
       </c>
-      <c r="L51" s="3"/>
-      <c r="M51" s="3"/>
-      <c r="N51" s="3"/>
-      <c r="O51" s="3"/>
-      <c r="P51" s="3"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="B52" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" s="3" t="s">
+      <c r="B52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="D52" s="3" t="s">
+      <c r="D52" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="E52" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="F52" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G52" s="3" t="s">
+      <c r="F52" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G52" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="H52" s="7" t="n">
+      <c r="H52" s="8" t="n">
         <v>0.76</v>
       </c>
-      <c r="I52" s="7" t="n">
+      <c r="I52" s="8" t="n">
         <f aca="false">B52*H52</f>
         <v>0.76</v>
       </c>
-      <c r="J52" s="7"/>
-      <c r="K52" s="7" t="n">
+      <c r="J52" s="8"/>
+      <c r="K52" s="8" t="n">
         <f aca="false">B52*J52</f>
         <v>0</v>
       </c>
-      <c r="L52" s="3"/>
-      <c r="M52" s="3"/>
-      <c r="N52" s="3"/>
-      <c r="O52" s="3"/>
-      <c r="P52" s="3"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="B53" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" s="3" t="s">
+      <c r="B53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D53" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E53" s="3" t="s">
+      <c r="E53" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="F53" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G53" s="3" t="s">
+      <c r="F53" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G53" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="H53" s="7" t="n">
+      <c r="H53" s="8" t="n">
         <v>1.06</v>
       </c>
-      <c r="I53" s="7" t="n">
+      <c r="I53" s="8" t="n">
         <f aca="false">B53*H53</f>
         <v>1.06</v>
       </c>
-      <c r="J53" s="7"/>
-      <c r="K53" s="7" t="n">
+      <c r="J53" s="8"/>
+      <c r="K53" s="8" t="n">
         <f aca="false">B53*J53</f>
         <v>0</v>
       </c>
-      <c r="L53" s="3"/>
-      <c r="M53" s="3"/>
-      <c r="N53" s="3"/>
-      <c r="O53" s="3"/>
-      <c r="P53" s="3"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B54" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D54" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E54" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="F54" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G54" s="3" t="s">
+      <c r="F54" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="H54" s="7" t="n">
+      <c r="H54" s="8" t="n">
         <v>1.38</v>
       </c>
-      <c r="I54" s="7" t="n">
+      <c r="I54" s="8" t="n">
         <f aca="false">B54*H54</f>
         <v>4.14</v>
       </c>
-      <c r="J54" s="7"/>
-      <c r="K54" s="7" t="n">
+      <c r="J54" s="8"/>
+      <c r="K54" s="8" t="n">
         <f aca="false">B54*J54</f>
         <v>0</v>
       </c>
-      <c r="L54" s="3"/>
-      <c r="M54" s="3"/>
-      <c r="N54" s="3"/>
-      <c r="O54" s="3"/>
-      <c r="P54" s="3"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="4"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="B55" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" s="3" t="s">
+      <c r="B55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D55" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E55" s="3" t="s">
+      <c r="E55" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="F55" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G55" s="8" t="s">
+      <c r="F55" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G55" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="H55" s="7" t="n">
+      <c r="H55" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="I55" s="7" t="n">
+      <c r="I55" s="8" t="n">
         <f aca="false">B55*H55</f>
         <v>0.1</v>
       </c>
-      <c r="J55" s="7"/>
-      <c r="K55" s="7" t="n">
+      <c r="J55" s="8"/>
+      <c r="K55" s="8" t="n">
         <f aca="false">B55*J55</f>
         <v>0</v>
       </c>
-      <c r="L55" s="3"/>
-      <c r="M55" s="3"/>
-      <c r="N55" s="3"/>
-      <c r="O55" s="3"/>
-      <c r="P55" s="3"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+      <c r="P55" s="4"/>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="B56" s="3" t="n">
+      <c r="B56" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="D56" s="3" t="s">
+      <c r="D56" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="E56" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="F56" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G56" s="8" t="s">
+      <c r="F56" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G56" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="H56" s="7" t="n">
+      <c r="H56" s="8" t="n">
         <v>0.13</v>
       </c>
-      <c r="I56" s="7" t="n">
+      <c r="I56" s="8" t="n">
         <f aca="false">B56*H56</f>
         <v>0.52</v>
       </c>
-      <c r="J56" s="7"/>
-      <c r="K56" s="7" t="n">
+      <c r="J56" s="8"/>
+      <c r="K56" s="8" t="n">
         <f aca="false">B56*J56</f>
         <v>0</v>
       </c>
-      <c r="L56" s="3"/>
-      <c r="M56" s="3"/>
-      <c r="N56" s="3"/>
-      <c r="O56" s="3"/>
-      <c r="P56" s="3"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="4"/>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="B57" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" s="3" t="s">
+      <c r="B57" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="D57" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E57" s="8" t="s">
+      <c r="E57" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="F57" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G57" s="8" t="s">
+      <c r="F57" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G57" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="H57" s="7" t="n">
+      <c r="H57" s="8" t="n">
         <v>10.63</v>
       </c>
-      <c r="I57" s="7" t="n">
+      <c r="I57" s="8" t="n">
         <f aca="false">B57*H57</f>
         <v>10.63</v>
       </c>
-      <c r="J57" s="7"/>
-      <c r="K57" s="7" t="n">
+      <c r="J57" s="8"/>
+      <c r="K57" s="8" t="n">
         <f aca="false">B57*J57</f>
         <v>0</v>
       </c>
-      <c r="L57" s="3"/>
-      <c r="M57" s="3"/>
-      <c r="N57" s="3"/>
-      <c r="O57" s="3"/>
-      <c r="P57" s="3"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="B58" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="3" t="s">
+      <c r="B58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="D58" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E58" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="F58" s="3" t="s">
+      <c r="F58" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G58" s="3" t="s">
+      <c r="G58" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="H58" s="7" t="n">
+      <c r="H58" s="8" t="n">
         <v>0.76</v>
       </c>
-      <c r="I58" s="7" t="n">
+      <c r="I58" s="8" t="n">
         <f aca="false">B58*H58</f>
         <v>0.76</v>
       </c>
-      <c r="J58" s="7" t="n">
+      <c r="J58" s="8" t="n">
         <v>0.541</v>
       </c>
-      <c r="K58" s="7" t="n">
+      <c r="K58" s="8" t="n">
         <f aca="false">B58*J58</f>
         <v>0.541</v>
       </c>
-      <c r="L58" s="3"/>
-      <c r="M58" s="3"/>
-      <c r="N58" s="3"/>
-      <c r="O58" s="3"/>
-      <c r="P58" s="3"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="4"/>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="B59" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" s="3" t="s">
+      <c r="B59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="D59" s="3" t="s">
+      <c r="D59" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="E59" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="F59" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G59" s="3" t="s">
+      <c r="G59" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="H59" s="7" t="n">
+      <c r="H59" s="8" t="n">
         <v>0.22</v>
       </c>
-      <c r="I59" s="7" t="n">
+      <c r="I59" s="8" t="n">
         <f aca="false">B59*H59</f>
         <v>0.22</v>
       </c>
-      <c r="J59" s="7" t="n">
+      <c r="J59" s="8" t="n">
         <v>0.14975</v>
       </c>
-      <c r="K59" s="7" t="n">
+      <c r="K59" s="8" t="n">
         <f aca="false">B59*J59</f>
         <v>0.14975</v>
       </c>
-      <c r="L59" s="3"/>
-      <c r="M59" s="3"/>
-      <c r="N59" s="3"/>
-      <c r="O59" s="3"/>
-      <c r="P59" s="3"/>
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
+      <c r="P59" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Updated files from video stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-02/P1012202501-BOM V2.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/Hardware/P1012202501-ESP32_Stepper_Controller/Project Outputs for P1012202501-02/P1012202501-BOM V2.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="10" documentId="11_4485A3C861C4F1C5C768334FD99282772C82B40A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC4F7823-ED5B-4326-B5B1-09D218575E6D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="-26700" yWindow="1845" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="P1012202501-ESP32_Stepper_Contr" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>